<commit_message>
progress: 10 village workbooks (sivaramans-llin 2026-10-08T18:30:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Amithamangalam_13.398978_80.050917.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Amithamangalam_13.398978_80.050917.xlsx
@@ -902,6 +902,11 @@
           <t>39</t>
         </is>
       </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3, 4, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -909,6 +914,11 @@
           <t>4</t>
         </is>
       </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -916,6 +926,11 @@
           <t>40</t>
         </is>
       </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2, 3, 4A, 4B1, 4B2, 4C, 5A1, 5A2, 5B, 5C, 6</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -923,6 +938,11 @@
           <t>41</t>
         </is>
       </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 4C, 4D1, 4D2</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -930,6 +950,11 @@
           <t>42</t>
         </is>
       </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 11C, 12, 13, 14, 2, 3, 4, 5, 6A, 6B, 6C, 6D, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -937,6 +962,11 @@
           <t>43</t>
         </is>
       </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -944,6 +974,11 @@
           <t>44</t>
         </is>
       </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 10C, 10D, 10E, 10F, 10G, 10H, 10I1, 10I2, 10J, 10K1, 10K2, 10L, 2A, 2B, 3A, 3B, 4, 5, 6, 7, 8A, 8B, 8C, 9</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -951,6 +986,11 @@
           <t>45</t>
         </is>
       </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13A, 13B, 14A, 14B, 14C, 14D, 15A, 15B, 16, 17, 18A, 18B, 19, 2, 20A, 20B, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -958,6 +998,11 @@
           <t>46</t>
         </is>
       </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 1A, 1B, 1C, 2, 20, 21, 3, 4, 5, 6, 7, 8A, 8B, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -965,6 +1010,11 @@
           <t>47</t>
         </is>
       </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>1, 2, 3A1, 3A2, 3B, 3C, 3D, 4A, 4B, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -972,6 +1022,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -979,6 +1034,11 @@
           <t>49</t>
         </is>
       </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A1, 4A2, 4A3, 4B1, 4B2, 4B3, 4C, 5A, 5B, 5C, 6</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -986,6 +1046,11 @@
           <t>5</t>
         </is>
       </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17A, 17B, 17C, 18, 19, 2, 3, 4, 5, 6A, 6B, 6C, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -993,6 +1058,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A, 12B, 13, 14, 15, 16, 17, 2A, 2B, 3, 4A, 4B, 5, 6, 7A, 7B, 7C, 8A, 8B, 8C, 9A, 9B, 9C, 9D</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1000,6 +1070,11 @@
           <t>51</t>
         </is>
       </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A, 12B, 12C, 12D, 2, 3, 4, 5, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1007,6 +1082,11 @@
           <t>52</t>
         </is>
       </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 2A, 2B, 3A, 3B, 3C, 4A1, 4A2, 4A3, 4B1, 4B2, 4B3, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1014,6 +1094,11 @@
           <t>53</t>
         </is>
       </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 1A, 1B, 1C, 2, 3A, 3B, 3C, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1021,6 +1106,11 @@
           <t>54</t>
         </is>
       </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16A, 16B, 17, 18A, 18B, 18C, 19, 2, 3, 4A, 4B, 4C, 5A, 5B, 5C, 6A, 6B, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1028,6 +1118,11 @@
           <t>55</t>
         </is>
       </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 2, 3A, 3B, 4, 5, 6, 7A, 7B, 8A, 8B, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1035,6 +1130,11 @@
           <t>56</t>
         </is>
       </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1A4, 1B1, 1B2, 1B3, 1C1, 1C2, 1C3, 2A, 2B1, 2B2, 2B3, 2C1, 2C2, 2D, 2E1, 2E2, 2F, 2G1, 2G2, 2H, 2I1, 2I2</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1042,6 +1142,11 @@
           <t>57</t>
         </is>
       </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>1A, 1B1A, 1B1B, 1B1C, 1B1D, 1B1E, 1B2, 2, 3, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1049,6 +1154,11 @@
           <t>58</t>
         </is>
       </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 11C, 12, 13, 14, 15, 16, 2, 3, 4, 5, 6, 7A, 7B, 8A, 8B, 8C, 9</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1056,6 +1166,11 @@
           <t>59</t>
         </is>
       </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3A, 3B, 3C, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1063,6 +1178,11 @@
           <t>6</t>
         </is>
       </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14A, 14B1, 14B2, 14C, 15A, 15B, 15C, 16, 17, 18, 19, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1070,6 +1190,11 @@
           <t>60</t>
         </is>
       </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>10A, 10B, 11, 12, 1A, 1B, 2, 3, 4A, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1077,6 +1202,11 @@
           <t>61</t>
         </is>
       </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2, 3, 4, 5A, 5B, 5C, 6A, 6B, 6C, 7</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1084,6 +1214,11 @@
           <t>62</t>
         </is>
       </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 1G, 1H, 1I, 1J, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1091,6 +1226,11 @@
           <t>63</t>
         </is>
       </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 2, 3, 4, 5, 6, 7A, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1098,6 +1238,11 @@
           <t>64</t>
         </is>
       </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15A, 15B, 16A, 16B, 17, 18A, 18B, 19, 2, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 3, 30, 31, 32, 33, 34, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1105,6 +1250,11 @@
           <t>65</t>
         </is>
       </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16A, 16B, 17, 18, 19, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1112,6 +1262,11 @@
           <t>66</t>
         </is>
       </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 3C, 3D, 3E, 3F, 3G, 3H, 4, 5, 6, 7, 8A, 8B, 8C</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -1119,6 +1274,11 @@
           <t>67</t>
         </is>
       </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -1126,6 +1286,11 @@
           <t>68</t>
         </is>
       </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -1133,6 +1298,11 @@
           <t>69</t>
         </is>
       </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -1140,6 +1310,11 @@
           <t>7</t>
         </is>
       </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16A, 16B, 17, 18, 19, 2, 20, 21, 22, 23, 3, 4, 5, 6, 7, 8, 9A, 9B, 9C</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -1147,6 +1322,11 @@
           <t>70</t>
         </is>
       </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -1154,6 +1334,11 @@
           <t>71</t>
         </is>
       </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -1161,6 +1346,11 @@
           <t>72</t>
         </is>
       </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -1168,6 +1358,11 @@
           <t>73</t>
         </is>
       </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -1175,6 +1370,11 @@
           <t>74</t>
         </is>
       </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -1182,6 +1382,11 @@
           <t>75</t>
         </is>
       </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -1189,6 +1394,11 @@
           <t>76</t>
         </is>
       </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -1196,6 +1406,11 @@
           <t>77</t>
         </is>
       </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17A, 17B, 17C, 18, 19, 2, 20, 21, 22, 3A, 3B, 3C, 4, 5, 6, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -1203,6 +1418,11 @@
           <t>78</t>
         </is>
       </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 3, 4, 5, 6A, 6B, 7, 8A, 8B, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -1210,6 +1430,11 @@
           <t>79</t>
         </is>
       </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 11C, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22A, 22B, 22C, 23, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -1217,6 +1442,11 @@
           <t>8</t>
         </is>
       </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 2, 3, 4, 5, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -1224,6 +1454,11 @@
           <t>80</t>
         </is>
       </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3, 4A, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -1231,6 +1466,11 @@
           <t>81</t>
         </is>
       </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2, 3, 4, 5, 6, 7A, 7B1, 7B2, 7C</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -1238,6 +1478,11 @@
           <t>82</t>
         </is>
       </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -1245,6 +1490,11 @@
           <t>83</t>
         </is>
       </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -1252,6 +1502,11 @@
           <t>84</t>
         </is>
       </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -1259,6 +1514,11 @@
           <t>85</t>
         </is>
       </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -1266,6 +1526,11 @@
           <t>86</t>
         </is>
       </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -1273,6 +1538,11 @@
           <t>87</t>
         </is>
       </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -1280,6 +1550,11 @@
           <t>88</t>
         </is>
       </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -1287,6 +1562,11 @@
           <t>89</t>
         </is>
       </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -1294,6 +1574,11 @@
           <t>9</t>
         </is>
       </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A, 12B, 13, 14, 15, 16, 17, 2A, 2B, 2C1, 2C2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -1301,6 +1586,11 @@
           <t>90</t>
         </is>
       </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -1308,6 +1598,11 @@
           <t>91</t>
         </is>
       </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>10, 1A, 1B, 1C, 1D, 1E, 1F, 2, 3A, 3B, 3C, 4, 5, 6A, 6B, 6C, 6D, 6E, 6F, 6G, 7, 8A, 8B, 8C, 8D, 9</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -1315,6 +1610,11 @@
           <t>92</t>
         </is>
       </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>10, 11, 1A, 1B, 1C, 1D, 1E, 2, 3, 4, 5A, 5B, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -1322,6 +1622,11 @@
           <t>93</t>
         </is>
       </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 4C, 5</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -1329,6 +1634,11 @@
           <t>94</t>
         </is>
       </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -1336,6 +1646,11 @@
           <t>95</t>
         </is>
       </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11, 12A, 12B, 12C, 13, 14, 15A, 15B, 2, 3, 4, 5, 6A, 6B, 6C, 6D, 7A, 7B, 7C, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -1343,6 +1658,11 @@
           <t>96</t>
         </is>
       </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -1350,6 +1670,11 @@
           <t>97</t>
         </is>
       </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -1357,11 +1682,21 @@
           <t>98</t>
         </is>
       </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2, 3, 4, 5, 6, 7A, 7B, 7C, 7D, 7E, 7F, 7G, 7H, 7I, 8</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
           <t>99</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>10A, 10B, 1A, 1B, 1C, 2, 3A, 3B, 3C, 3D, 3E, 3F, 3G, 3H, 3I, 3J, 3K, 3L, 3M, 3N, 3O, 4, 5, 6, 7, 8, 9</t>
         </is>
       </c>
     </row>

</xml_diff>